<commit_message>
refactor: remove hardcoded synergy fallback, add color field from config table
- Delete ~50 lines hardcoded synergy fallback data in SynergyManager.LoadSynergyData

- Fix color bug: tag switch used Chinese keys but config uses English tags, all colors were white

- Add ColorHex field to SynergyConfig + parse in ConfigLoader

- Add color column to synergy.xlsx, export to JSON
</commit_message>
<xml_diff>
--- a/Project/tables/data/synergy.xlsx
+++ b/Project/tables/data/synergy.xlsx
@@ -468,7 +468,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I8"/>
+  <dimension ref="A1:J8"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -528,6 +528,11 @@
           <t>array_str</t>
         </is>
       </c>
+      <c r="J1" t="inlineStr">
+        <is>
+          <t>string</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" s="2" t="inlineStr">
@@ -575,6 +580,11 @@
           <t>范围加成%(|分隔)</t>
         </is>
       </c>
+      <c r="J2" t="inlineStr">
+        <is>
+          <t>羁绊颜色</t>
+        </is>
+      </c>
     </row>
     <row r="3">
       <c r="A3" s="3" t="inlineStr">
@@ -620,6 +630,11 @@
       <c r="I3" s="3" t="inlineStr">
         <is>
           <t>range_bonus</t>
+        </is>
+      </c>
+      <c r="J3" t="inlineStr">
+        <is>
+          <t>color</t>
         </is>
       </c>
     </row>
@@ -663,6 +678,11 @@
           <t>0|0</t>
         </is>
       </c>
+      <c r="J4" t="inlineStr">
+        <is>
+          <t>e6b34d</t>
+        </is>
+      </c>
     </row>
     <row r="5">
       <c r="A5" s="5" t="n">
@@ -704,6 +724,11 @@
           <t>0|10</t>
         </is>
       </c>
+      <c r="J5" t="inlineStr">
+        <is>
+          <t>4de680</t>
+        </is>
+      </c>
     </row>
     <row r="6">
       <c r="A6" s="4" t="n">
@@ -745,6 +770,11 @@
           <t>0|0</t>
         </is>
       </c>
+      <c r="J6" t="inlineStr">
+        <is>
+          <t>e66633</t>
+        </is>
+      </c>
     </row>
     <row r="7">
       <c r="A7" s="5" t="n">
@@ -786,6 +816,11 @@
           <t>20|50</t>
         </is>
       </c>
+      <c r="J7" t="inlineStr">
+        <is>
+          <t>804de6</t>
+        </is>
+      </c>
     </row>
     <row r="8">
       <c r="A8" s="4" t="n">
@@ -825,6 +860,11 @@
       <c r="I8" s="4" t="inlineStr">
         <is>
           <t>0|0</t>
+        </is>
+      </c>
+      <c r="J8" t="inlineStr">
+        <is>
+          <t>994d1a</t>
         </is>
       </c>
     </row>

</xml_diff>